<commit_message>
Restructure Paik works spreadsheet to assignment format with market-value evidence
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DsnrAXHBSv8Rwd8VRMcuBt
</commit_message>
<xml_diff>
--- a/백남준_대표작_20선.xlsx
+++ b/백남준_대표작_20선.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20선" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="출처" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="시장 비교사례" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="출처" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'20선'!$A$1:$K$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'20선'!$A$1:$N$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,6 +33,7 @@
       <name val="맑은 고딕"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="맑은 고딕"/>
@@ -41,6 +43,11 @@
       <name val="맑은 고딕"/>
       <i val="1"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
   <fills count="3">
@@ -82,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -94,7 +101,13 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -461,20 +474,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="52" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
-    <col width="6" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -500,35 +516,50 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>구분</t>
+          <t>① 개요·특징</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>재료·매체</t>
+          <t>② 재료·기법·표현양식</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>내용·특징</t>
+          <t>③-1 미술사적 가치</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>소장처/발표</t>
+          <t>③-2 시장가치 (사용자 원본 수치)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>③-3 시장가치 근거 등급</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>③-4 비교·산정 메모</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>④ 작품상태·프로비넌스(소장·발표)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>검증</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>원본 대비 정정·비고</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>정정·비고</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>기존 10선</t>
         </is>
@@ -555,35 +586,50 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>싱글채널 필름(플럭서스)</t>
+          <t>플럭서스 시기의 필름 작품. 영사 시 필름 자체의 먼지·흠집이 드러나는 구조(내용 설명은 기존 지식)</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>16mm 흑백 무음 필름, 약 8분</t>
+          <t>싱글채널 필름(플럭서스) / 16mm 흑백 무음 필름, 약 8분</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>플럭서스 시기의 필름 작품. 영사 시 필름 자체의 먼지·흠집이 드러나는 구조(내용 설명은 기존 지식)</t>
+          <t>플럭서스의 '비움' 미학과 영화 매체의 물질성을 드러낸 초기 작업</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
+          <t>(원본에 없음)</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>해당 작품의 공개 낙찰 사례를 찾지 못함. 시트 '시장 비교사례'의 유사 작품 거래가로 간접 참고</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
           <t>배급: EAI(Electronic Arts Intermix)</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>△</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>원본 표의 'CRT 모니터' 서술은 오류(필름 작품). 1960s 행에 둔 것은 적절</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -610,35 +656,50 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>참여형 TV 작품</t>
+          <t>관객 소리·조작이 화면 영상을 변형시키는 참여형 TV 작품. 1960s 관객 참여 작품 계열로 분류됨</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>TV 수상기, 마이크 입력 등</t>
+          <t>참여형 TV 작품 / TV 수상기, 마이크 입력 등</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>관객 소리·조작이 화면 영상을 변형시키는 참여형 TV 작품. 1960s 관객 참여 작품 계열로 분류됨</t>
+          <t>수용자의 참여를 TV 수상기 조작으로 구현한 초기 사례</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
+          <t>(원본에 없음)</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>해당 작품의 공개 낙찰 사례를 찾지 못함. 시트 '시장 비교사례'의 유사 작품 거래가로 간접 참고</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
           <t>1963 Galerie Parnass 전시(기존 지식)</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>△</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>세부 구성·소장처는 추가 확인 필요</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -665,35 +726,50 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>사운드 설치</t>
+          <t>1963년 부퍼탈 Galerie Parnass 'Exposition of Music–Electronic Television'에서 발표(전시 정보는 기존 지식). 관객이 직접 소리를 '무작위 접근'하는 참여형 작품</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>벽에 붙인 오디오 테이프를 손에 든 헤드로 읽어 재생</t>
+          <t>사운드 설치 / 벽에 붙인 오디오 테이프를 손에 든 헤드로 읽어 재생</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>1963년 부퍼탈 Galerie Parnass 'Exposition of Music–Electronic Television'에서 발표(전시 정보는 기존 지식). 관객이 직접 소리를 '무작위 접근'하는 참여형 작품</t>
+          <t>관객이 직접 소리에 접근하는 참여형 사운드 작품</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
+          <t>(원본에 없음)</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>해당 작품의 공개 낙찰 사례를 찾지 못함. 시트 '시장 비교사례'의 유사 작품 거래가로 간접 참고</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
           <t>Tate Liverpool/FACT 2010 전시 출품 확인</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>△</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>연도 표기가 출처마다 다름(1963 / 1963–79)</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -720,35 +796,50 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>로봇/퍼포먼스 조각</t>
+          <t>1964년 뉴욕 아방가르드 페스티벌 초연으로 알려짐(Tate는 1965 부퍼탈 24 Stunden으로 기술 → 불일치). 1982 휘트니 회고전 기간 매디슨가에서 퍼포먼스 중 차에 치임(운전자: William Anastasi). 2019 Tate Modern 전시 출품</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>20채널 원격조종 로봇(일본 엔지니어 협업), 오디오 장치 등</t>
+          <t>로봇/퍼포먼스 조각 / 20채널 원격조종 로봇(일본 엔지니어 협업), 오디오 장치 등</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>1964년 뉴욕 아방가르드 페스티벌 초연으로 알려짐(Tate는 1965 부퍼탈 24 Stunden으로 기술 → 불일치). 1982 휘트니 회고전 기간 매디슨가에서 퍼포먼스 중 차에 치임(운전자: William Anastasi). 2019 Tate Modern 전시 출품</t>
+          <t>로봇을 퍼포먼스의 주체로 세워 기계와 인간의 관계를 유머로 다룬 초기 작업</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
+          <t>US$150만~200만(레플리카 거래가)</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>경매 최고가(약 US$131만) 초과 → 근거 필요. 해당 작품의 공개 낙찰 사례를 찾지 못함. 시트 '시장 비교사례'의 유사 작품 거래가로 간접 참고</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
           <t>소장처 미확정(1982년 당시 독일 소장품 대여로 보도)</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>△</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>원본 오류: '1982 MoMA 회고전'→휘트니미술관. '구겐하임 소장'은 근거 없음. '최초의 예술가'는 과장. 시장가치 근거 없음</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -775,35 +866,50 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>TV 조각</t>
+          <t>자석이 전자빔을 왜곡해 화면 이미지를 변형. 뉴욕 첫 개인전 출품작</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>17인치 흑백 TV + 대형 산업용 자석</t>
+          <t>TV 조각 / 17인치 흑백 TV + 대형 산업용 자석</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>자석이 전자빔을 왜곡해 화면 이미지를 변형. 뉴욕 첫 개인전 출품작</t>
+          <t>TV 이미지를 물리적으로 변형하는 초기 미디어 조각, 관객 개입 구조</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
+          <t>US$100만</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. 공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
           <t>Whitney Museum (acc. 86.60) / 다른 버전: 백남준아트센터(1965/69)</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>원본의 '1965 Howard Wise Gallery' 전시는 근거 없음(첫 뉴욕 개인전으로 확인되며 화랑명은 Galeria Bonino로 알고 있으나 재확인 권장). '관객이 자석을 움직임'은 참여형이라는 설명과 부합</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -830,35 +936,50 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>TV 설치</t>
+          <t>달을 가장 오래된 빛의 매체로 보고 TV 화면에 달의 위상을 구현</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>TV 수상기 다수</t>
+          <t>TV 설치 / TV 수상기 다수</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>달을 가장 오래된 빛의 매체로 보고 TV 화면에 달의 위상을 구현</t>
+          <t>자연의 빛(달)과 전자 매체를 겹친 동양적 사유</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
+          <t>(원본에 없음)</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
           <t>백남준아트센터 소장품 카탈로그</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>재제작 연도(2000)가 병기됨</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -885,35 +1006,50 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>퍼포먼스 오브제</t>
+          <t>샬롯 무어먼의 첫 TV Cello 연주는 1971 뉴욕 Bonino Gallery(EAI 기록). 영상 송출 시스템 구성은 기존 지식</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>TV 3대를 쌓고 현을 장착</t>
+          <t>퍼포먼스 오브제 / TV 3대를 쌓고 현을 장착</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>샬롯 무어먼의 첫 TV Cello 연주는 1971 뉴욕 Bonino Gallery(EAI 기록). 영상 송출 시스템 구성은 기존 지식</t>
+          <t>퍼포머의 몸과 매체를 결합한 무어먼 협업 대표작</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
+          <t>US$70만</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. 공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
           <t>Walker Art Center (acc. 1992.6.1-.10)</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="M8" s="3" t="inlineStr">
         <is>
           <t>원본 오류: '1971 Avant-Garde Festival 초연'→Bonino Gallery. '모먼/샬롯 무어만'→샬롯 무어먼(Charlotte Moorman)으로 통일</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -940,35 +1076,50 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>싱글채널 비디오</t>
+          <t>1974.1 WNET(뉴욕)에서 첫 방송. 다문화 퍼포먼스·음악 영상 콜라주. TV Garden에서 이 영상을 사용(Tate 확인). 존 고드프리 공동작업·백-아베 합성기 사용은 기존 지식</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>컬러 비디오테이프, 약 28분</t>
+          <t>싱글채널 비디오 / 컬러 비디오테이프, 약 28분</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>1974.1 WNET(뉴욕)에서 첫 방송. 다문화 퍼포먼스·음악 영상 콜라주. TV Garden에서 이 영상을 사용(Tate 확인). 존 고드프리 공동작업·백-아베 합성기 사용은 기존 지식</t>
+          <t>비디오아트가 방송에 진입한 초기 사례, 글로벌 TV에 대한 비전</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
+          <t>US$50만</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. 해당 작품의 공개 낙찰 사례를 찾지 못함. 시트 '시장 비교사례'의 유사 작품 거래가로 간접 참고</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
           <t>WNET 방송 / 배급 EAI</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>△</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="M9" s="3" t="inlineStr">
         <is>
           <t>원본 오류: '다채널 영상'→싱글채널. '우리는 곧 글로벌 TV 시대에…' 따옴표 인용은 원문 불일치(실제는 '지구상 어느 방송이든 채널을 돌릴 수 있고 TV 가이드가 맨해튼 전화번호부만큼 두꺼워질 것'). 시장가치 근거 없음</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -995,35 +1146,50 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>CCTV 설치</t>
+          <t>불상이 자신의 실시간 영상을 응시하는 폐쇄회로 구조. 여러 버전 존재(Tate/FACT 2010 전시에 7점)</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>불상 + CCTV 카메라 + 모니터</t>
+          <t>CCTV 설치 / 불상 + CCTV 카메라 + 모니터</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>불상이 자신의 실시간 영상을 응시하는 폐쇄회로 구조. 여러 버전 존재(Tate/FACT 2010 전시에 7점)</t>
+          <t>동양 종교 도상과 서구 기술 매체의 대비</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
+          <t>US$100만~150만</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. 해당 작품의 공개 낙찰 사례를 찾지 못함. 시트 '시장 비교사례'의 유사 작품 거래가로 간접 참고</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
           <t>버전별 상이(미확인)</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>△</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="M10" s="3" t="inlineStr">
         <is>
           <t>원본의 '20여 점 버전'·'MoMA·Tate·MMCA 소장'은 미확인. 1960s 행에 둔 것은 오류(1974)</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1050,35 +1216,50 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>비디오 설치</t>
+          <t>자연과 기술의 공존. Tate 2019 전시 오프닝 작품(1974/2002)</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>실제 식물 + TV 모니터(구겐하임 버전 약 150대·식물 약 500그루), Global Groove 영상 송출</t>
+          <t>비디오 설치 / 실제 식물 + TV 모니터(구겐하임 버전 약 150대·식물 약 500그루), Global Groove 영상 송출</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>자연과 기술의 공존. Tate 2019 전시 오프닝 작품(1974/2002)</t>
+          <t>자연과 기술의 공존을 다룬 설치, 다수 버전으로 재제작</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
+          <t>US$80만 이상</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. 공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
           <t>Guggenheim(2000 버전, International Directors Council 기증)</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t>원본 '구겐하임·NJP 상설전시'는 구겐하임만 확인. 연도는 1974 / 1974–77 / 2002 등 표기 혼재</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1105,35 +1286,50 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>비디오 설치</t>
+          <t>작은 물고기가 화면 사이를 헤엄치는 천장 설치 작품</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>천장 설치, 88개 화면에 물고기 영상</t>
+          <t>비디오 설치 / 천장 설치, 88개 화면에 물고기 영상</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>작은 물고기가 화면 사이를 헤엄치는 천장 설치 작품</t>
+          <t>천장 설치형 다채널 영상 작품</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
+          <t>(원본에 없음)</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
           <t>Museum Kunstpalast, Düsseldorf (inv. ZM1985.6)</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
+      <c r="M12" s="3" t="inlineStr">
         <is>
           <t>연도가 출처마다 다름</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1160,31 +1356,46 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>비디오 설치</t>
+          <t>1982 휘트니 회고전을 위해 제작. 록 음악 vs 한국 전통 가락, 피라미드의 견고함 vs 영상의 흐름 등 대립 구도</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>TV 40대를 피라미드로 쌓음</t>
+          <t>비디오 설치 / TV 40대를 피라미드로 쌓음</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>1982 휘트니 회고전을 위해 제작. 록 음악 vs 한국 전통 가락, 피라미드의 견고함 vs 영상의 흐름 등 대립 구도</t>
+          <t>피라미드 구조에 대립 요소를 병치한 비디오 조각</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
+          <t>(원본에 없음)</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
           <t>Whitney Museum (acc. 82.11)</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="M13" s="3" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1211,35 +1422,50 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>위성 생중계</t>
+          <t>1984.1.1 방송. 오웰의 『1984』에 대한 응답. 진행: George Plimpton. 미국 PBS 방송. 대서양 위성 연결이 불안정해 미국·프랑스에서 서로 다른 버전이 방영됨</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>위성 생방송 (뉴욕 WNET–파리 퐁피두센터 + 독일·한국 방송사)</t>
+          <t>위성 생중계 / 위성 생방송 (뉴욕 WNET–파리 퐁피두센터 + 독일·한국 방송사)</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>1984.1.1 방송. 오웰의 『1984』에 대한 응답. 진행: George Plimpton. 미국 PBS 방송. 대서양 위성 연결이 불안정해 미국·프랑스에서 서로 다른 버전이 방영됨</t>
+          <t>국제 위성 생중계를 예술 매체로 사용한 대표 사례</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
+          <t>(원본에 없음)</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>산정 불가</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>위성 생중계는 실물 거래 대상이 아님. 시가 대신 영상 원본(테이프) 가치·문화적 가치로 서술하는 것이 타당</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
           <t>WNET / Centre Pompidou 외</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="M14" s="3" t="inlineStr">
         <is>
           <t>시청자 약 2,500만 명은 홍보·백과 자료에서 반복되는 근사치(국가별 근거 미확인). '방송미술 사상 최초' 단정은 피할 것</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1266,35 +1492,50 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>비디오 설치</t>
+          <t>TV 모니터로 만든 미국 국기. 여러 버전 존재</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>TV 모니터 다수로 구성한 성조기 (DIA 버전: Quasar 10인치 84대, 3채널 컬러 영상, 레이저디스크)</t>
+          <t>비디오 설치 / TV 모니터 다수로 구성한 성조기 (DIA 버전: Quasar 10인치 84대, 3채널 컬러 영상, 레이저디스크)</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>TV 모니터로 만든 미국 국기. 여러 버전 존재</t>
+          <t>대중적 이미지(국기)를 비디오 모니터로 재해석</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
+          <t>(원본에 없음)</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
           <t>Detroit Institute of Arts (Video Flag x, 1986 구입) / Hirshhorn Museum (1985–96 표기)</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="M15" s="3" t="inlineStr">
         <is>
           <t>버전별로 연도·구성이 다름</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1321,35 +1562,50 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>위성 생중계</t>
+          <t>서울 아시안게임 시기에 맞춘 동서 대화 프로젝트. 뉴욕 진행: Dick Cavett, 도쿄 진행: 사카모토 류이치. 1986년 가을 미국 PBS 방영</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>뉴욕–서울–도쿄 3원 위성 연결, 3시간 방송</t>
+          <t>위성 생중계 / 뉴욕–서울–도쿄 3원 위성 연결, 3시간 방송</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>서울 아시안게임 시기에 맞춘 동서 대화 프로젝트. 뉴욕 진행: Dick Cavett, 도쿄 진행: 사카모토 류이치. 1986년 가을 미국 PBS 방영</t>
+          <t>동서 간 위성 대화를 기획한 3원 생중계</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
+          <t>US$60만</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>산정 불가</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. 위성 생중계는 실물 거래 대상이 아님. 시가 대신 영상 원본(테이프) 가치·문화적 가치로 서술하는 것이 타당</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
           <t>제작: WNET(뉴욕), KBS, Asahi National Broadcasting (EAI 기록)</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="M16" s="3" t="inlineStr">
         <is>
           <t>원본 오류: 'NHK'→아사히 내셔널 브로드캐스팅. 시장가치 US 60만 달러는 근거 없음(방송 이벤트는 거래 대상이 아님). 일부 카탈로그의 1988 표기는 오류로 판단</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1376,35 +1632,50 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>위성 생중계</t>
+          <t>한국·미국·브라질·오스트리아·독일·아일랜드·이스라엘·일본·이탈리아·중국·영국·소련 등 12개국 연결(Tate). 서울올림픽 연계는 기존 지식</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>국제 위성 방송</t>
+          <t>위성 생중계 / 국제 위성 방송</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>한국·미국·브라질·오스트리아·독일·아일랜드·이스라엘·일본·이탈리아·중국·영국·소련 등 12개국 연결(Tate). 서울올림픽 연계는 기존 지식</t>
+          <t>12개국을 연결한 위성 생중계, 위성 3부작의 완결편</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
+          <t>(원본에 없음)</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>산정 불가</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>위성 생중계는 실물 거래 대상이 아님. 시가 대신 영상 원본(테이프) 가치·문화적 가치로 서술하는 것이 타당</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
           <t>Tate 전시 자료</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>△</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="M17" s="3" t="inlineStr">
         <is>
           <t>원본 목록에 누락된 위성 3부작의 완결편</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1431,35 +1702,50 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>비디오 타워 설치</t>
+          <t>2018.2 가동 중단 → 3개년 보존·복원 → 2022.9.15 재가동. 수리·교체 대수는 보도별로 상이(735대 수리·268대 LCD / 737대 중고 수급·266대 LCD), 영상 8종 디지털 변환. 주 4일·하루 2시간 가동(잠정)</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>CRT 모니터 1,003대 + 철골 구조, 높이 18.5m</t>
+          <t>비디오 타워 설치 / CRT 모니터 1,003대 + 철골 구조, 높이 18.5m</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>2018.2 가동 중단 → 3개년 보존·복원 → 2022.9.15 재가동. 735대 수리, 상단 268대는 LCD 교체, 영상 8종 디지털 변환. 주 4일·하루 2시간 가동(잠정)</t>
+          <t>한국 현대미술의 대표 설치이자 CRT 작품 보존·복원 논의의 중심 사례</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
+          <t>US$1천만 이상(추정)</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>경매 최고가(약 US$131만) 초과 → 근거 필요. 공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
           <t>국립현대미술관 과천관 중앙홀</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>원본 오류: '2023 복원 완료'→재가동은 2022.9.15(백서는 2023 발간 예정). '로비'→과천관 중앙홀. 1990s 행에 둔 것은 오류(1988). 시장가치 US 1천만 달러 근거 없음</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>원본 오류: '2023 복원 완료'→재가동은 2022.9.15(백서는 2023 발간 예정). '로비'→과천관 중앙홀. 1990s 행에 둔 것은 오류(1988). 시장가치 US 1천만 달러 근거 없음 복원 대수는 기사마다 달라 MMCA 백서로 재확인 필요.</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1486,35 +1772,50 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>멀티 프로젝션 설치</t>
+          <t>1993 베니스비엔날레 독일관(한스 하케와 공동, 황금사자상)에서 발표(기존 지식). 2019 Tate Modern에서 재현</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>프로젝터 34대 (Tate 재현 기준)</t>
+          <t>멀티 프로젝션 설치 / 프로젝터 34대 (Tate 재현 기준)</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>1993 베니스비엔날레 독일관(한스 하케와 공동, 황금사자상)에서 발표(기존 지식). 2019 Tate Modern에서 재현</t>
+          <t>베니스비엔날레 독일관 출품 대형 프로젝션 설치</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
+          <t>(원본에 없음)</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>해당 작품의 공개 낙찰 사례를 찾지 못함. 시트 '시장 비교사례'의 유사 작품 거래가로 간접 참고</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
           <t>Tate Modern 2019–20 전시 확인</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>△</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr">
+      <c r="M19" s="3" t="inlineStr">
         <is>
           <t>Venice 1993 정보는 추가 출처 확인 권장</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1541,35 +1842,50 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>비디오 월 설치</t>
+          <t>글로벌 정보 네트워크에 대한 예견. 철골 프레임 설치</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>모니터 + 맞춤 비디오월 시스템, 287×380×80cm</t>
+          <t>비디오 월 설치 / 모니터 + 맞춤 비디오월 시스템, 287×380×80cm</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>글로벌 정보 네트워크에 대한 예견. 철골 프레임 설치</t>
+          <t>네트워크 사회에 대한 예견을 담은 비디오월</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
+          <t>(원본에 없음)</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
           <t>ZKM | Karlsruhe</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr">
+      <c r="M20" s="3" t="inlineStr">
         <is>
           <t>원본의 '2001'은 오류. Tate는 1993, ZKM 등은 1994로 표기하여 출처별 상이</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1596,35 +1912,50 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>비디오 설치</t>
+          <t>네온으로 그린 미국 지도에 주(州)별 영상. 인터스테이트 고속도로·케이블TV·초기 인터넷과 연결</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>51채널 비디오, 네온, 맞춤 전자장치, 강철·목재, 약 15×40×4 ft</t>
+          <t>비디오 설치 / 51채널 비디오, 네온, 맞춤 전자장치, 강철·목재, 약 15×40×4 ft</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>네온으로 그린 미국 지도에 주(州)별 영상. 인터스테이트 고속도로·케이블TV·초기 인터넷과 연결</t>
+          <t>정보고속도로 담론을 네온·영상으로 시각화한 대형 설치</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
+          <t>US$500만(보험가)</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>직접 거래 사례 없음</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>경매 최고가(약 US$131만) 초과 → 근거 필요. 공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
           <t>Smithsonian American Art Museum (acc. 2002.23, Gift of the artist)</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="J21" s="3" t="inlineStr">
+      <c r="M21" s="3" t="inlineStr">
         <is>
           <t>원본 오류: 'SAAM 커미션'→작가 기증. TV '300대'는 미확인(공식 기록은 51채널). '생전 최대 규모'는 다다익선과 충돌. 보험가 US 500만·NFT/LED 리마스터링 논의는 근거 없음</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1633,26 +1964,19 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>검증 표기: O = 웹 출처로 확인 / △ = 일부만 확인(나머지는 기존 지식, 인용 전 재확인 권장)</t>
+          <t>시장가치 원본 수치는 사용자가 이전에 조사한 값이며, 이번 검색에서 근거를 확인하지 못했습니다(그대로 보존, 판단은 '③-3/③-4' 참고).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>시장가치는 신뢰할 공개 근거를 찾지 못해 모두 제외했습니다. 필요하면 경매 낙찰가·보험가 등 출처가 있는 값만 별도 기재하세요.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>연도순 정렬. '기존 10선'=Y는 사용자 원본에 있던 10개 작품.</t>
+          <t>검증: O=웹 출처로 확인 / △=일부 확인(나머지는 기존 지식, 인용 전 재확인).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K21"/>
+  <autoFilter ref="A1:N21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1663,7 +1987,310 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>비교 작품</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>제작연도</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>경매일(연도)</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>경매사</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>결과</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>집계처</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>Rocketship to Virtual Venus</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>미상</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>China Guardian (베이징)</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>US$1,312,770 (MutualArt 집계 최고가)</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>MutualArt</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>https://www.mutualart.com/Artist/Nam-June-Paik/BC44AEA7A8F9403E</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Wright Brothers</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>미상(조각)</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Christie's 홍콩</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>HK$5,031,500 ≈ US$646,897</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>artnet</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>https://news.artnet.com/market/nam-june-paiks-estate-joins-gagosians-empire-324451</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Stag</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>1996</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Seoul Auction 홍콩</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>낙찰 HK$460만 ≈ 6.6억 원 ≈ US$59만 (일부 국내 기사는 '590만 달러'로 보도 → 통화 오기로 판단)</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Korea Times / 시사위클리</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>https://www.koreatimes.co.kr/lifestyle/arts-theater/20170529/paiks-stag-breaks-auction-record</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>(Christie's 최고 낙찰)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>미상</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>미상</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Christie's 2018-05-26</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>HK$4,540,000 ≈ US$578,757</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>LotSearch</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>https://www.lotsearch.net/artist/nam-june-paik</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Enlightenment Compressed</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>1994</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>미상</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Phillips</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>US$107,100 (수수료 포함 여부 미확인)</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Phillips</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>https://phillips.com/detail/nam-june-paik/NY010821/191</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>MT-TV (4인치 TV 작품)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>미상</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Ravenel 홍콩</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>HK$264,000 ≈ US$33,890</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Ravenel</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>https://ravenel.com/en/cata/lotsIn/f932b614-5bff-42cb-a8cf-664dce64cff5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>※ 집계 사이트·언론 수치이며 경매사 원 기록으로 교차 확인하지 않았습니다. 환율은 보도된 환산값을 그대로 인용.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>※ 위 사례는 모두 소형·중형 작품 또는 에디션 작품으로, 대형 설치·공공 소장품(다다익선 등)의 직접 비교 대상이 아닙니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>※ 과제에서 금액을 제시해야 한다면, 비교사례 기반 '추정'임과 산정 방식(비교사례법·원가법 등)을 함께 서술하는 것을 권장합니다.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1671,254 +2298,326 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>출처명</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Whitney 1982 회고전 보도자료(EAI)</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>https://www.eai.org/user_files/supporting_documents/Paik_Retrospective at Whitney_1982.pdf</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Tate – When the future was now</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>https://www.tate.org.uk/tate-etc/issue-21-spring-2011/when-future-was-now</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>SAAM – Electronic Superhighway</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>https://www.si.edu/object/saam_2002.23</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Walker – TV Cello</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>https://walkerart.org/collections/artworks/tv-cello</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Whitney – Magnet TV</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>https://whitney.org/collection/works/6139</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Whitney – V-yramid</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>https://whitney.org/collection/works/5459</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>EAI – Bye Bye Kipling</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>https://eai.org/title.htm?id=1933</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Video Out – Bye Bye Kipling</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>https://videoout.ca/catalog/bye-bye-kipling</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Cinematheque KOFA – Bye Bye Kipling</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>https://eng.koreafilm.or.kr/movie/PM_010610</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Wikipedia – Good Morning, Mr. Orwell</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Good_Morning,_Mr._Orwell</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>TV Garden (Variable Media)</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>https://www.variablemedia.net/pdf/TV_Garden.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Global Groove (UT Landmarks)</t>
         </is>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>https://landmarks.utexas.edu/video-art/global-groove</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Tate Modern 2019 전시 가이드</t>
         </is>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>https://www.tate.org.uk/whats-on/tate-modern/nam-june-paik/exhibition-guide</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Tate Liverpool 2010 전시</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>https://www.tate.org.uk/whats-on/tate-liverpool/exhibition/nam-june-paik</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>DIA – Video Flag x</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>https://dia.org/collection/video-flag-x-56329</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>Kunstpalast – Fish Flies on Sky</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>https://sammlung.kunstpalast.de/en/objects/details/41591</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>ZKM – Nam June Paik</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>https://zkm.de/en/node/7877</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>백남준아트센터 – Moon is the Oldest TV</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>https://prenjpac-en.ggcf.kr/?p=701</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>아주경제 – 다다익선 재가동(2022.9)</t>
         </is>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>https://www.ajunews.com/view/20220915175111038</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>EAI – Paik 작품 목록</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>https://www.eai.org/artists/481</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Korea Times – Stag 낙찰</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>https://www.koreatimes.co.kr/lifestyle/arts-theater/20170529/paiks-stag-breaks-auction-record</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>시사위클리 – 백남준 최고가 보도</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>https://www.sidae.com/article/2017082516108028204</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>MutualArt – Nam June Paik</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>https://www.mutualart.com/Artist/Nam-June-Paik/BC44AEA7A8F9403E</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>LotSearch – Nam June Paik</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>https://www.lotsearch.net/artist/nam-june-paik</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Phillips – Enlightenment Compressed</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>https://phillips.com/detail/nam-june-paik/NY010821/191</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>Ravenel 2010 HK</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>https://ravenel.com/en/cata/lotsIn/f932b614-5bff-42cb-a8cf-664dce64cff5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace boilerplate valuation memos with per-work verified findings
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DsnrAXHBSv8Rwd8VRMcuBt
</commit_message>
<xml_diff>
--- a/백남준_대표작_20선.xlsx
+++ b/백남준_대표작_20선.xlsx
@@ -611,7 +611,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>해당 작품의 공개 낙찰 사례를 찾지 못함. 시트 '시장 비교사례'의 유사 작품 거래가로 간접 참고</t>
+          <t>EAI 배급 필름 작품으로 개별 낙찰 사례를 찾지 못함. 참고: 같은 시기 에디션 판화(Novecento 석판화, 1992)가 약 US$12,583(Millon 2015)에 낙찰</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>해당 작품의 공개 낙찰 사례를 찾지 못함. 시트 '시장 비교사례'의 유사 작품 거래가로 간접 참고</t>
+          <t>개별 낙찰·구입 사례를 찾지 못함(초기 TV 작품은 미술관 소장 중심)</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>해당 작품의 공개 낙찰 사례를 찾지 못함. 시트 '시장 비교사례'의 유사 작품 거래가로 간접 참고</t>
+          <t>개별 낙찰 사례를 찾지 못함. 참고: 소형 에디션 TV 작품(MT-TV, 1994)이 HK$264,000(Ravenel 2010)에 낙찰</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>경매 최고가(약 US$131만) 초과 → 근거 필요. 해당 작품의 공개 낙찰 사례를 찾지 못함. 시트 '시장 비교사례'의 유사 작품 거래가로 간접 참고</t>
+          <t>경매 최고가(약 US$131만) 초과 → 근거 필요. 1964 원형은 1982년 이후 대여·전시 위주로 거래 사례 없음. 참고(유사 로봇 계열): Sotheby's 2017 'Video Robot' 추정가 US$6만~8만(낙찰가 미확인), Sotheby's 홍콩 2016 'Robot'(1993) 추정가 HK$50만~70만(낙찰가 미확인), 'Circuit Bored'(1994) US$207,900(Masterworks 집계, 미검증)</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. 공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. Whitney가 구입(Dieter Rosenkranz 기금, acc. 86.60), 구입가는 비공개. 다른 버전은 백남준아트센터 소장. 경매 낙찰 사례 없음</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+          <t>백남준아트센터 소장(모니터 13대 버전). 거래·낙찰 사례 없음</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. 공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. Walker Art Center 소장(Otto Piene·Elizabeth Goldring 구소장, acc. 1992.6.1-.10). 국내 보도에 대구은행 소장 버전이 언급됨(단일 출처). 경매 낙찰 사례 없음</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. 해당 작품의 공개 낙찰 사례를 찾지 못함. 시트 '시장 비교사례'의 유사 작품 거래가로 간접 참고</t>
+          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. 테이프 단독 거래 사례를 찾지 못함. 참고: 1984년 'Global Groove' 응용 설치가 Lempertz에서 추정가 €20만~30만으로 출품(낙찰가 미확인)</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. 해당 작품의 공개 낙찰 사례를 찾지 못함. 시트 '시장 비교사례'의 유사 작품 거래가로 간접 참고</t>
+          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. 같은 제목의 낙찰 사례는 찾지 못함. 참고(불상 모티프 작품): 'Enlightenment Compressed'(1994) US$107,100(Phillips, 추정 US$4만~6만), 'Neon Buddha'(1997) £63,000(Phillips), 'Baby Buddha' HK$230만(Christie's 홍콩 2007, Artprice)</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
@@ -1241,7 +1241,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. 공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. Guggenheim 소장(International Directors Council 기증)으로 구입가가 없음. 경매 사례 없음</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+          <t>Museum Kunstpalast 소장(inv. ZM1985.6). 경매 낙찰 사례를 찾지 못함</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+          <t>Whitney가 Lemberg Foundation 기금으로 구입(acc. 82.11), 구입가는 비공개. 경매 사례 없음</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
@@ -1447,7 +1447,7 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>위성 생중계는 실물 거래 대상이 아님. 시가 대신 영상 원본(테이프) 가치·문화적 가치로 서술하는 것이 타당</t>
+          <t>위성 방송 이벤트로 매매 대상이 아님. 영상 기록물 가치로만 서술 가능</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+          <t>DIA가 1986년 Founders Society 기금으로 구입, Hirshhorn은 Holenia Purchase Fund로 1996년 구입. 두 곳 모두 구입가 비공개, 경매 낙찰 사례 못 찾음</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
@@ -1587,7 +1587,7 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. 위성 생중계는 실물 거래 대상이 아님. 시가 대신 영상 원본(테이프) 가치·문화적 가치로 서술하는 것이 타당</t>
+          <t>경매 최고가 범위 내이나 해당 작품의 직접 거래 근거 없음. 위성 방송 이벤트로 매매 대상이 아님. 영상 기록물 가치로만 서술 가능</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>위성 생중계는 실물 거래 대상이 아님. 시가 대신 영상 원본(테이프) 가치·문화적 가치로 서술하는 것이 타당</t>
+          <t>위성 방송 이벤트로 매매 대상이 아님. 영상 기록물 가치로만 서술 가능</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>경매 최고가(약 US$131만) 초과 → 근거 필요. 공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+          <t>경매 최고가(약 US$131만) 초과 → 근거 필요. 국립현대미술관 소장 비매품으로 거래 사례 없음. 3개년 보존·복원 사업이 시행됐으나 총비용은 확인 못함. 보험가·평가액 미확인(정보공개청구 대상)</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>해당 작품의 공개 낙찰 사례를 찾지 못함. 시트 '시장 비교사례'의 유사 작품 거래가로 간접 참고</t>
+          <t>개별 거래·낙찰 사례를 찾지 못함</t>
         </is>
       </c>
       <c r="K19" s="3" t="inlineStr">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+          <t>ZKM 소장. 개별 거래·낙찰 사례를 찾지 못함</t>
         </is>
       </c>
       <c r="K20" s="3" t="inlineStr">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>경매 최고가(약 US$131만) 초과 → 근거 필요. 공공 소장품. 비교 사례(시트 '시장 비교사례')의 간접 참고만 가능. 보험가는 비공개가 일반적(정보공개청구 대상)</t>
+          <t>경매 최고가(약 US$131만) 초과 → 근거 필요. SAAM에 작가 기증(2002.23)이라 구입가가 없음. 보험가·평가액 미확인(Smithsonian 정보공개 대상)</t>
         </is>
       </c>
       <c r="K21" s="3" t="inlineStr">
@@ -1987,7 +1987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2224,56 +2224,278 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
+          <t>Baby Buddha</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>미상</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Christie's 홍콩</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>HK$230만 (Artprice 인용)</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Artprice</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>https://www.artprice.com/artmarketinsight/video-art-the-moving-image</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Neon Buddha</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>미상</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Phillips</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>£63,000 (추정 £5만~7만)</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Phillips</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>https://www.phillips.com/detail/白南準/146592</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Video Robot</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>미상</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Sotheby's</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>추정 US$6만~8만 (낙찰가 미확인)</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Sotheby's</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>https://sothebys.com/en/auctions/ecatalogue/2017/contemporary-art-day-auction-n09762/lot.436.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Robot</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Sotheby's 홍콩</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>추정 HK$50만~70만 (낙찰가 미확인)</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Sotheby's</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>https://sothebys.com/en/auctions/ecatalogue/2016/boundless-contemporary-art-hk0651/lot.524.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Global Groove 응용 설치</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>1984</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>미상</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Lempertz 쾰른</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>추정 €20만~30만 (낙찰가 미확인)</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Lempertz</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>https://www.lempertz.com/en/press/lempertz-to-auction-video-art-by-nam-june-paik-from-the-collection-of-wulf-herzogenrath.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Circuit Bored</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>1994</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Christie's</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>US$207,900 (Masterworks 집계, 미검증)</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Masterworks</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>https://www.masterworks.com/academy/artists/nam-june-paik</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
           <t>MT-TV (4인치 TV 작품)</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>미상</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>2010</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Ravenel 홍콩</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>HK$264,000 ≈ US$33,890</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Ravenel</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>https://ravenel.com/en/cata/lotsIn/f932b614-5bff-42cb-a8cf-664dce64cff5</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>※ 집계 사이트·언론 수치이며 경매사 원 기록으로 교차 확인하지 않았습니다. 환율은 보도된 환산값을 그대로 인용.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>※ 위 사례는 모두 소형·중형 작품 또는 에디션 작품으로, 대형 설치·공공 소장품(다다익선 등)의 직접 비교 대상이 아닙니다.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>※ 과제에서 금액을 제시해야 한다면, 비교사례 기반 '추정'임과 산정 방식(비교사례법·원가법 등)을 함께 서술하는 것을 권장합니다.</t>
         </is>

</xml_diff>